<commit_message>
Preserve local people updates after merging remote master
</commit_message>
<xml_diff>
--- a/assets/files/home_show.xlsx
+++ b/assets/files/home_show.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AAA_AutoI_Lab\assets\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{422FF14D-E13B-4765-94D2-2291CEFFD1AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647D159F-59B6-4684-8206-EB4A845B6FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1350" yWindow="2160" windowWidth="22830" windowHeight="11220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -506,7 +506,7 @@
     <hyperlink ref="B6" r:id="rId5" xr:uid="{C469C7EA-89D5-4202-84CE-675418FEDAD0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
 

</xml_diff>